<commit_message>
fixup! validate and normalize quiz structure on upload; show errors on main menu
</commit_message>
<xml_diff>
--- a/tests/files/basic.xlsx
+++ b/tests/files/basic.xlsx
@@ -9,7 +9,6 @@
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Tabelle2" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="92">
   <si>
     <t xml:space="preserve">Monatsrückblick</t>
   </si>
@@ -299,86 +298,18 @@
   </si>
   <si>
     <t xml:space="preserve">Stratford-upon-Avon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Über 6000 Meter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nicht über 6000 Meter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elbrus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Denali (6190)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mont Blanc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerro Aconcagua (6960)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cotopaxi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monte Pissis (6793)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Misty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Makalu (8463)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sliabh Ard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annapurna 1 (8091)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altas Montagnona</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nanga Parbat (8125)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Secret Peak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pico Veintimilla (6228)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pik Vysoka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Island Peak (6189)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kastanjeblomst Tinde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hidden Peak (8068)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kibo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pik Pobeda (7439)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/\ mmm"/>
-    <numFmt numFmtId="167" formatCode="0\ %"/>
-    <numFmt numFmtId="168" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,97 +348,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <u val="single"/>
-      <sz val="20"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <u val="single"/>
-      <sz val="18"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="20"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="20"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="18"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="18"/>
-      <color rgb="FF1B1E25"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor rgb="FF33CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.3999"/>
-        <bgColor rgb="FF99CCFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -542,11 +389,9 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -563,7 +408,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -575,7 +420,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -595,78 +440,6 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -676,66 +449,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFA9D18E"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00B0F0"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF1B1E25"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -747,37 +460,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -5882,259 +5595,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="10.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="80.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="43.14"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12"/>
-      <c r="B1" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="D1" s="15"/>
-      <c r="E1" s="16"/>
-    </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="16"/>
-    </row>
-    <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-    </row>
-    <row r="4" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="16"/>
-    </row>
-    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16"/>
-    </row>
-    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-    </row>
-    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-    </row>
-    <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-    </row>
-    <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-    </row>
-    <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="15"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="16"/>
-    </row>
-    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16"/>
-    </row>
-    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
-    </row>
-    <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="16"/>
-    </row>
-    <row r="17" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="27"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-    </row>
-    <row r="18" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16"/>
-    </row>
-    <row r="19" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-    </row>
-    <row r="20" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-    </row>
-    <row r="21" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>